<commit_message>
fix: align Phase 1 sample data with INR demo
</commit_message>
<xml_diff>
--- a/data/commercial_ops_data.xlsx
+++ b/data/commercial_ops_data.xlsx
@@ -28,7 +28,7 @@
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="3">
     <numFmt numFmtId="164" formatCode="YYYY-MM-DD HH:MM:SS"/>
-    <numFmt numFmtId="165" formatCode="&quot;$&quot;#,##0.00"/>
+    <numFmt numFmtId="165" formatCode="&quot;₹&quot;#,##0.00"/>
     <numFmt numFmtId="166" formatCode="yyyy-mm-dd"/>
   </numFmts>
   <fonts count="3">
@@ -2184,7 +2184,7 @@
         <v>46236</v>
       </c>
       <c r="D20" s="4" t="n">
-        <v>46266</v>
+        <v>46295</v>
       </c>
       <c r="E20" s="5" t="n">
         <v>52000</v>
@@ -2473,7 +2473,7 @@
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>ACH</t>
+          <t>NEFT</t>
         </is>
       </c>
     </row>
@@ -2496,7 +2496,7 @@
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>ACH</t>
+          <t>NEFT</t>
         </is>
       </c>
     </row>
@@ -2588,7 +2588,7 @@
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>ACH</t>
+          <t>NEFT</t>
         </is>
       </c>
     </row>

</xml_diff>